<commit_message>
Marchio YMCA Prime Sport Club e nome «YMCA Prime Training»
Logo vettorializzato (assets/logo.svg) e usato in benvenuto e schermata di avvio;
icone rigenerate con il triangolo rosso del marchio. Palette dell'app dal logo:
rosso #E21D23, bianco e grafite (giorni scheda, avatar e gruppi muscolari compresi).
Nome app, demo, README e checklist store aggiornati; codice palestra di prova PRIME.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dkgg7PSUWnhATau7aG1SC2
</commit_message>
<xml_diff>
--- a/docs/Preventivo_Schede_Palestra.xlsx
+++ b/docs/Preventivo_Schede_Palestra.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="183">
   <si>
-    <t xml:space="preserve">Schede palestra · canone mensile e avvio</t>
+    <t xml:space="preserve">YMCA Prime Training · canone mensile e avvio</t>
   </si>
   <si>
     <t xml:space="preserve">Celle blu = ipotesi da modificare (giallo = da decidere o confermare). Nero = formule. Il canone dipende soprattutto dal tempo di assistenza, non dal numero di soci.</t>
@@ -172,7 +172,7 @@
     <t xml:space="preserve">Esclusi: Apple Developer (99 €/anno) e Google Play (25 € una tantum), che vanno intestati alla palestra (vedi foglio Confronto). IVA esclusa.</t>
   </si>
   <si>
-    <t xml:space="preserve">Schede palestra · stima del carico sul database</t>
+    <t xml:space="preserve">YMCA Prime Training · stima del carico sul database</t>
   </si>
   <si>
     <t xml:space="preserve">Celle blu = ipotesi da modificare (giallo = da confermare con la palestra). Nero = formule.</t>

</xml_diff>